<commit_message>
Update deck: 2025 data, ASEAN-10 scope, slide reorg, remove Excel from tracking
- Growth rates updated to 2025 (IMF/national stats agencies)
- Regional figures switched to ASEAN-10: GDP $4.2T, population ~690M, 5th largest economy
- All "ASEAN-6" labels replaced with "Southeast Asia"
- GDP bar chart reordered (SEA now above Japan)
- Digital economy $263B -> $300B+, e-commerce $114.6B -> $185B
- AI infra aligned to $30B+ in H1 2024 (Google/Temasek/Bain source)
- Germany median age corrected 45.3 -> 45.7
- Slide 6 country cards redistributed to Slides 3/4/5
- Slide 5 rearranged to 2-column layout with horizontal stat cards
- Slide 6 hero bar restyled, charts enlarged, callout updated
- Removed SEA Facts.xlsx from git tracking

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEA Facts.xlsx
+++ b/SEA Facts.xlsx
@@ -576,14 +576,14 @@
     <row r="1" ht="18.5" customHeight="1" s="9">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>LANMEA CAPITAL - Definitive Southeast Asia Fact Bank (ASEAN-6)</t>
+          <t>LANMEA CAPITAL - Definitive Southeast Asia Fact Bank</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Indonesia, Vietnam, Philippines, Thailand, Malaysia, Singapore. Consolidated from multiple research sources. March 2026.</t>
+          <t>Indonesia, Vietnam, Philippines, Thailand, Malaysia, Singapore + Myanmar, Cambodia, Laos, Brunei for aggregate figures. Consolidated from IMF, World Bank, UN, Bain/Google/Temasek, and primary sources.</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>THE BLOC THAT RIVALS AN ECONOMY - ASEAN as a single force</t>
+          <t>THE BLOC THAT RIVALS AN ECONOMY - Southeast Asia as a single force</t>
         </is>
       </c>
     </row>
@@ -644,17 +644,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ASEAN-6 is the world's 6th largest economy - on track to surpass Japan by 2030</t>
+          <t>Southeast Asia is the world's 5th largest economy - already larger than Japan</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Combined GDP: ~$3.8T (2024); projected $5.8T by 2030 (+53% growth in 6 years)</t>
+          <t>Combined GDP: ~$4.2T (2025, ASEAN-10); projected $6T+ by 2030</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Larger than UK ($3.5T); closing in on Japan ($4.1T); India ($4.3T) and Germany ($4.6T) above; will rival both by 2030</t>
+          <t>Larger than Japan ($4.1T) and UK ($3.5T); India ($4.3T) and Germany ($4.6T) above; on track to surpass Germany by end of decade</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -681,12 +681,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>614 million people across six economies - larger than the EU</t>
+          <t>~690 million people across Southeast Asia - larger than the EU</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Indonesia: 284M, Philippines: 116M, Vietnam: 101M, Thailand: 72M, Malaysia: 36M, Singapore: 6M</t>
+          <t>Indonesia: 284M, Philippines: 116M, Vietnam: 101M, Thailand: 72M, Myanmar: 55M, Malaysia: 36M, Cambodia: 17M, Laos: 8M, Singapore: 6M, Brunei: 0.5M</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1011,7 +1011,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>THE DIGITAL LEAP - A $263B internet economy that's now profitable</t>
+          <t>THE DIGITAL LEAP - A $300B+ internet economy that's now profitable</t>
         </is>
       </c>
     </row>
@@ -1028,12 +1028,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>SEA internet economy hit $263B GMV - 7.4x growth in a decade</t>
+          <t>SEA internet economy hit $300B+ GMV - 7.4x growth in a decade</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>$263B GMV (2024, +15% YoY); $89B revenue (+14%); $11B profit (+24%); on track for $305B in 2025</t>
+          <t>$300B+ GMV (2025, ASEAN-10); $11B profit (2024); previously $263B (2024, ASEAN-6)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>THE YOUTH DIVIDEND - 614M people, most of them young and working</t>
+          <t>THE YOUTH DIVIDEND - ~690M people, most of them young and working</t>
         </is>
       </c>
     </row>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Philippines: 25.7 | Malaysia: 30.1 | Indonesia: 30.2 | Vietnam: 32.9 | Thailand: 40.1 | Singapore: 38.4 — all younger than Germany (45.3) or Japan (49.4)</t>
+          <t>Philippines: 25.7 | Malaysia: 30.1 | Indonesia: 30.2 | Vietnam: 32.9 | Thailand: 40.1 | Singapore: 38.4 — all younger than Europe/Japan</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Germany: 45.3 | Japan: 49.4 | US: 38.3 | China: 39.6 | Even India (28.4) is close to ASEAN average</t>
+          <t>Germany: 45.7 | Japan: 49.4 | US: 38.3 | China: 39.6 | Even India (28.8) is close to SEA average</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>$50B+ in AI infrastructure investment poured into SEA since 2023</t>
+          <t>$30B+ committed to AI infrastructure in H1 2024 alone</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Microsoft, Google, Amazon investing heavily; AI market: $4B (2024) → $16B by 2033; 85% of SEA businesses use AI</t>
+          <t>Microsoft, Google, Amazon investing heavily; $30B+ in H1 2024 (Google/Temasek/Bain e-Conomy SEA 2024); AI market: $4B (2024) → $16B by 2033; 85% of SEA businesses use AI</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>7.1% growth (2024); FTSE upgrading to emerging market status 2026; manufacturing = 86% of exports</t>
+          <t>8.0% growth (2025); FTSE upgrading to emerging market status 2026; manufacturing = 86% of exports</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Median Age (2024)</t>
+          <t>Median Age (2025)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2850,35 +2850,25 @@
           <t>30.2</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>~30</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>24.3</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>28.5</t>
-        </is>
+      <c r="C4" s="2" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>30.1</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>42.8</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>28.4</t>
-        </is>
+      <c r="H4" s="2" t="n">
+        <v>28.8</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -2890,10 +2880,8 @@
           <t>38.3</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>45.3</t>
-        </is>
+      <c r="K4" s="2" t="n">
+        <v>45.7</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -3028,37 +3016,37 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GDP Growth (2024)</t>
+          <t>GDP Growth (2025)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>~2.5%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>5.2%</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>4.8%</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>4.1%</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -3772,7 +3760,7 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Sources: IMF WEO 2025, UN DESA 2024, Worldometer, Google/Temasek/Bain e-Conomy SEA 2024, ASEAN Investment Report 2024, World Bank, EF EPI</t>
+          <t>Sources: IMF WEO 2025, UN DESA 2024, Worldometer, Google/Temasek/Bain e-Conomy SEA 2025, ASEAN Investment Report 2024</t>
         </is>
       </c>
     </row>
@@ -3909,12 +3897,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>ASEAN-10 (including Myanmar, Cambodia, Laos, Brunei)</t>
+          <t>ASEAN-10 aggregate data exclusion (OVERRIDDEN)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Focus is ASEAN-6 where PE/VC activity actually exists; smaller markets add noise, not signal</t>
+          <t>Previously excluded; NOW INCLUDED for aggregate figures (GDP, population, digital economy). Country-level data still focuses on the 6 core economies where PE/VC activity exists. Updated April 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>